<commit_message>
updated excel file for all tools
</commit_message>
<xml_diff>
--- a/CMPT470_M3_Results.xlsx
+++ b/CMPT470_M3_Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/age159_usask_ca/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A39DD2BA-D139-4A32-B5CD-D0D7ED16ED36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE63EFB8-8C53-4825-9072-1C9DDA86FB1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="348" yWindow="2172" windowWidth="7500" windowHeight="7392" xr2:uid="{7CF85045-BB3F-4D86-A7F1-99D2A27485AE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{7CF85045-BB3F-4D86-A7F1-99D2A27485AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="85">
   <si>
     <t>Tool Name</t>
   </si>
@@ -268,13 +268,37 @@
   </si>
   <si>
     <t>https://ieeexplore.ieee.org/document/10927826</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>tool executed correctly for given dataset</t>
+  </si>
+  <si>
+    <t>5000 samples</t>
+  </si>
+  <si>
+    <t>TES-B</t>
+  </si>
+  <si>
+    <t>AI-assisted research</t>
+  </si>
+  <si>
+    <t>the original results entered here are from the original paper, not from the alternative tool's paper. This tool required a few interventions but it did work in the end. It was mainly just parsing issues</t>
+  </si>
+  <si>
+    <t>~40k samples</t>
+  </si>
+  <si>
+    <t>https://github.com/jacobwwh/graphmatch_clone</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -301,7 +325,7 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -692,7 +716,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41B3B5F0-18C0-460A-AF22-6B3BF3536BEB}">
   <dimension ref="B2:S26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.85546875" customWidth="1"/>
     <col min="3" max="3" width="67.42578125" customWidth="1"/>
@@ -714,7 +738,7 @@
     <col min="19" max="19" width="37.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19">
+    <row r="2" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -770,7 +794,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:19" ht="28.9">
+    <row r="3" spans="2:19" ht="45" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>18</v>
       </c>
@@ -826,7 +850,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="2:19" ht="87">
+    <row r="4" spans="2:19" ht="90" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>33</v>
       </c>
@@ -863,11 +887,11 @@
       <c r="M4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="N4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>30</v>
+      <c r="N4" s="2">
+        <v>0.96</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0.98</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>30</v>
@@ -882,7 +906,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="2:19" ht="43.5">
+    <row r="5" spans="2:19" ht="45" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>45</v>
       </c>
@@ -938,7 +962,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="2:19" ht="101.25">
+    <row r="6" spans="2:19" ht="90" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>55</v>
       </c>
@@ -966,20 +990,35 @@
       <c r="J6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K6" s="2"/>
+      <c r="K6" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="L6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
+      <c r="M6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N6" s="2">
+        <v>0.93</v>
+      </c>
+      <c r="O6" s="2">
+        <v>0.93</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="R6" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="7" spans="2:19" ht="72.75">
+      <c r="S6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="2:19" ht="60" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>61</v>
       </c>
@@ -1035,7 +1074,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="2:19" ht="72.75">
+    <row r="8" spans="2:19" ht="45" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>71</v>
       </c>
@@ -1045,22 +1084,53 @@
       <c r="D8" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-    </row>
-    <row r="9" spans="2:19" ht="72.75">
+      <c r="E8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="2:19" ht="45" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>74</v>
       </c>
@@ -1070,22 +1140,53 @@
       <c r="D9" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-    </row>
-    <row r="10" spans="2:19">
+      <c r="E9" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="N9" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="O9" s="2">
+        <v>0.92</v>
+      </c>
+      <c r="P9" s="2">
+        <v>0.36</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="S9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -1104,7 +1205,7 @@
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
     </row>
-    <row r="11" spans="2:19">
+    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -1123,7 +1224,7 @@
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
     </row>
-    <row r="12" spans="2:19">
+    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -1142,7 +1243,7 @@
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
     </row>
-    <row r="13" spans="2:19">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -1161,7 +1262,7 @@
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
     </row>
-    <row r="14" spans="2:19">
+    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -1180,7 +1281,7 @@
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
     </row>
-    <row r="15" spans="2:19">
+    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -1199,7 +1300,7 @@
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
     </row>
-    <row r="16" spans="2:19">
+    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -1218,7 +1319,7 @@
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
     </row>
-    <row r="17" spans="2:18">
+    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -1237,7 +1338,7 @@
       <c r="Q17" s="2"/>
       <c r="R17" s="2"/>
     </row>
-    <row r="18" spans="2:18">
+    <row r="18" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -1256,7 +1357,7 @@
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
     </row>
-    <row r="19" spans="2:18">
+    <row r="19" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -1275,7 +1376,7 @@
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
     </row>
-    <row r="20" spans="2:18">
+    <row r="20" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -1294,7 +1395,7 @@
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
     </row>
-    <row r="21" spans="2:18">
+    <row r="21" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -1313,7 +1414,7 @@
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
     </row>
-    <row r="22" spans="2:18">
+    <row r="22" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -1332,7 +1433,7 @@
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
     </row>
-    <row r="23" spans="2:18">
+    <row r="23" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -1351,7 +1452,7 @@
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
     </row>
-    <row r="24" spans="2:18">
+    <row r="24" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -1370,7 +1471,7 @@
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
     </row>
-    <row r="25" spans="2:18">
+    <row r="25" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -1389,7 +1490,7 @@
       <c r="Q25" s="2"/>
       <c r="R25" s="2"/>
     </row>
-    <row r="26" spans="2:18">
+    <row r="26" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -1420,12 +1521,31 @@
     <hyperlink ref="E5" r:id="rId8" xr:uid="{EB0310E5-E2E6-44E1-B9BF-6963AE41C5F9}"/>
     <hyperlink ref="E6" r:id="rId9" xr:uid="{DE720DDD-E156-48E4-B5A0-23688EBBDB78}"/>
     <hyperlink ref="E7" r:id="rId10" xr:uid="{2AD7492B-4EA0-445E-9B91-E83E76CFA142}"/>
+    <hyperlink ref="E9" r:id="rId11" xr:uid="{63893BFD-8352-45C2-89C8-C87484819CE1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId12"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="4ddce786-d625-4fa5-9e38-f614bafba860" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000C756C11F3385C47A1E6DCE92772F821" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="462d258f5ca36bef57646e43ccf9df58">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="4ddce786-d625-4fa5-9e38-f614bafba860" xmlns:ns4="82ddf94a-5f4c-4a2f-8a30-8937e89abf39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68201432d5583b0182a337230d54ebd9" ns3:_="" ns4:_="">
     <xsd:import namespace="4ddce786-d625-4fa5-9e38-f614bafba860"/>
@@ -1652,31 +1772,39 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="4ddce786-d625-4fa5-9e38-f614bafba860" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9CF30D4-9387-4E53-90BC-F158C5F3B87E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E915839-0ABC-4C8D-A48D-7A27EF5E2D00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{521721C7-DC93-46BB-904D-22E3629FDD72}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{521721C7-DC93-46BB-904D-22E3629FDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4ddce786-d625-4fa5-9e38-f614bafba860"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E915839-0ABC-4C8D-A48D-7A27EF5E2D00}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9CF30D4-9387-4E53-90BC-F158C5F3B87E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4ddce786-d625-4fa5-9e38-f614bafba860"/>
+    <ds:schemaRef ds:uri="82ddf94a-5f4c-4a2f-8a30-8937e89abf39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>